<commit_message>
fix: repair field deployment templates and excel import
</commit_message>
<xml_diff>
--- a/templates/reports/슬러지사진대지.xlsx
+++ b/templates/reports/슬러지사진대지.xlsx
@@ -1,35 +1,123 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\OneDrive\바탕 화면\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B02D551-8C66-4C84-9EA3-F5D58D4BA9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-5970" windowWidth="29040" windowHeight="15720" xr2:uid="{2D54B54E-E300-40D9-A72B-BEBEF89EADFB}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="템플릿" state="visible" r:id="rId4"/>
+    <sheet name="사진대지" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="날짜1">사진대지!$A$4</definedName>
+    <definedName name="날짜2">사진대지!$A$7</definedName>
+    <definedName name="반출량1">사진대지!$C$6</definedName>
+    <definedName name="반출량2">사진대지!$C$9</definedName>
+    <definedName name="사진1">사진대지!$B$4</definedName>
+    <definedName name="사진2">사진대지!$B$7</definedName>
+    <definedName name="필증1">사진대지!$D$4</definedName>
+    <definedName name="필증2">사진대지!$D$7</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
-    <t>슬러지사진대지 기본 템플릿</t>
+    <t>슬러지 반출</t>
   </si>
   <si>
-    <t>이 파일은 기본 번들 템플릿입니다. 실제 양식은 필요에 따라 교체해주세요.</t>
+    <t>청소필증</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사 진 대 지</t>
+  </si>
+  <si>
+    <t>날 짜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>슬러지 반출 사진대지</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +128,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -48,15 +136,291 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="19">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -72,9 +436,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -112,7 +476,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -184,7 +548,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -216,16 +580,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -347,67 +715,98 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F43E93-A065-4714-8799-CDC031B67305}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="12.3984375" customWidth="1"/>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="20.59765625" customWidth="1"/>
+    <col min="4" max="4" width="29.296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:4" ht="44.4" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="12" t="s">
+        <v>4</v>
       </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="3" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="13"/>
+      <c r="D3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
+    <row r="4" spans="1:4" ht="120.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" spans="1:4" ht="120.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="14"/>
+      <c r="B6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" spans="1:4" ht="120.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="5"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="9"/>
+    </row>
+    <row r="8" spans="1:4" ht="120.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" spans="1:4" ht="54.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="7"/>
+      <c r="B9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <mergeCells count="10">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:C8"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.88" right="0.7" top="1.28" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>